<commit_message>
Add more to techniques matrix and results matrix
</commit_message>
<xml_diff>
--- a/Research/TheProjectKaggle/TheFinalCode/result matrix.xlsx
+++ b/Research/TheProjectKaggle/TheFinalCode/result matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shwes\Projects\Thesis\Research\TheProjectKaggle\TheFinalCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD54D8D8-1F76-41C4-8FFF-BF023F9DC5F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C329635-64EC-4BAE-95CE-2D3D81EE9F5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,17 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="48">
   <si>
     <t>Technique</t>
   </si>
   <si>
-    <t>Train Score</t>
-  </si>
-  <si>
-    <t>Eval Score</t>
-  </si>
-  <si>
     <t>Theoretical best possible</t>
   </si>
   <si>
@@ -96,9 +90,6 @@
     <t>Estimated Workload</t>
   </si>
   <si>
-    <t>Done</t>
-  </si>
-  <si>
     <t>Research time</t>
   </si>
   <si>
@@ -130,13 +121,61 @@
   </si>
   <si>
     <t>&lt;1 hour + debugging  + above</t>
+  </si>
+  <si>
+    <t>Val Loss</t>
+  </si>
+  <si>
+    <t>Done (2 hours ish)</t>
+  </si>
+  <si>
+    <t>1-2 hours</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>3rd place's qwen judge with one model</t>
+  </si>
+  <si>
+    <t>""</t>
+  </si>
+  <si>
+    <t>debugging</t>
+  </si>
+  <si>
+    <t>Eval chrf</t>
+  </si>
+  <si>
+    <t>Eval BLEU</t>
+  </si>
+  <si>
+    <t>Eval combined</t>
+  </si>
+  <si>
+    <t>Unknown, lots, research</t>
+  </si>
+  <si>
+    <t>Kaggle  Private</t>
+  </si>
+  <si>
+    <t>Kaggle  Public</t>
+  </si>
+  <si>
+    <t>Kaggle Translations Examples</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>4 epochs may have overfit</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -151,8 +190,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -165,8 +209,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -194,19 +244,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -487,186 +551,309 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I21"/>
-  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:S22"/>
+  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="21" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="66.3984375" customWidth="1"/>
-    <col min="2" max="2" width="17.19921875" customWidth="1"/>
-    <col min="5" max="9" width="22.9296875" customWidth="1"/>
+    <col min="2" max="3" width="27.46484375" customWidth="1"/>
+    <col min="10" max="14" width="22.9296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:19" ht="21" customHeight="1">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+    </row>
+    <row r="2" spans="1:19" ht="21" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+    </row>
+    <row r="3" spans="1:19" ht="21" customHeight="1">
+      <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3">
+        <v>0.24215600000000001</v>
+      </c>
+      <c r="E3" s="6">
+        <v>25.804300000000001</v>
+      </c>
+      <c r="F3" s="6">
+        <v>26.073799999999999</v>
+      </c>
+      <c r="G3" s="5">
+        <v>43.78</v>
+      </c>
+      <c r="H3" s="5">
+        <v>64.180000000000007</v>
+      </c>
+      <c r="I3" s="7">
+        <v>53.01</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="21" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="1:19" ht="21" customHeight="1">
+      <c r="A5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="I5" s="6"/>
+    </row>
+    <row r="6" spans="1:19" ht="21" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" spans="1:19" ht="21" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="1:19" ht="21" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="1:19" ht="21" customHeight="1">
+      <c r="A9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" spans="1:19" ht="21" customHeight="1">
+      <c r="A10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-    </row>
-    <row r="2" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="I10" s="6"/>
+    </row>
+    <row r="11" spans="1:19" ht="21" customHeight="1">
+      <c r="A11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="I11" s="6"/>
+    </row>
+    <row r="12" spans="1:19" ht="21" customHeight="1">
+      <c r="A12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="I12" s="6"/>
+    </row>
+    <row r="13" spans="1:19" ht="21" customHeight="1">
+      <c r="A13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="I13" s="6"/>
+    </row>
+    <row r="14" spans="1:19" ht="21" customHeight="1">
+      <c r="A14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="I14" s="6"/>
+    </row>
+    <row r="15" spans="1:19" ht="21" customHeight="1">
+      <c r="A15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="I15" s="6"/>
+    </row>
+    <row r="16" spans="1:19" ht="21" customHeight="1">
+      <c r="A16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="I16" s="6"/>
+    </row>
+    <row r="17" spans="1:9" ht="21" customHeight="1">
+      <c r="A17" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="5" t="s">
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="I17" s="6"/>
+    </row>
+    <row r="18" spans="1:9" ht="21" customHeight="1">
+      <c r="A18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="I18" s="6"/>
+    </row>
+    <row r="19" spans="1:9" ht="21" customHeight="1">
+      <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="5" t="s">
+      <c r="B19" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="I19" s="6"/>
+    </row>
+    <row r="20" spans="1:9" ht="21" customHeight="1">
+      <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="7" t="s">
+      <c r="B20" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="5"/>
-      <c r="B20" s="3"/>
-    </row>
-    <row r="21" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="6"/>
-      <c r="B21" s="3"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="I20" s="6"/>
+    </row>
+    <row r="21" spans="1:9" ht="21" customHeight="1">
+      <c r="A21" s="3"/>
+    </row>
+    <row r="22" spans="1:9" ht="21" customHeight="1">
+      <c r="A22" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>